<commit_message>
v2.6: study_design 개정 + analysis_set 신열 + AF/RVR 엄격화 + HRV 제외 + SAE 통합
- study_design (N): 随机/随机分为/randomized 표현만 있어도 RCT 분류
  (배정방법 적절성은 RoB 2.0 D1에서 평가). 입원순서·번호순 등
  systematic non-random allocation은 non-RCT
- 신규 AU열 analysis_set (ITT/PP/NR 메타분석 분류 코드, mITT→ITT 통합)
  기존 notes는 AV로 이동 (47열 → 48열)
- af_type_other 코드 5 (AF with RVR) 기준 엄격화 — Methods/Inclusion에
  치료 전 안정시 HR ≥ 110 명시 시만
- HRV 및 파생 지표 (SDNN, RMSSD, LF, HF, DC, AC, Poincaré 등) 아웃컴 완전 제외
- SAE 통합 추출 (AE total과 동일 방식, 논문이 SAE로 묶어 보고한 경우만)
- 분류 모호 케이스는 6B 불확실 항목 의무 명시
- migrate_master_v2.6.py 신규 — v2.5.x → v2.6 마이그레이션 스크립트
  (멱등성·자동 백업·사후 검증). 위치: 00_skills/cpg-data-extraction/
- 매뉴얼 docx v2.6 신규, merge-skill v2.6 호환성 메모 추가
- sample_v2.6.xlsx 신설, master/example xlsx 48열 마이그레이션

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/90_Output/AF_CPG_data_extraction_example(2-39).xlsx
+++ b/90_Output/AF_CPG_data_extraction_example(2-39).xlsx
@@ -499,10 +499,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU13"/>
+  <dimension ref="A1:AV13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
-    <col width="30" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="30" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -738,6 +739,11 @@
       </c>
       <c r="AU1" s="5" t="inlineStr">
         <is>
+          <t>analysis_set</t>
+        </is>
+      </c>
+      <c r="AV1" s="5" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -956,6 +962,7 @@
         </is>
       </c>
       <c r="AU2" s="2" t="n"/>
+      <c r="AV2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1169,6 +1176,7 @@
         </is>
       </c>
       <c r="AU3" s="2" t="n"/>
+      <c r="AV3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1384,6 +1392,7 @@
         </is>
       </c>
       <c r="AU4" s="2" t="n"/>
+      <c r="AV4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1597,6 +1606,7 @@
         </is>
       </c>
       <c r="AU5" s="2" t="n"/>
+      <c r="AV5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1816,6 +1826,13 @@
 outcome 에 IQR 값 있음 -&gt; 변환필요</t>
         </is>
       </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>대규모 다기관 연구
+비교군이 placebo
+outcome 에 IQR 값 있음 -&gt; 변환필요</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2031,6 +2048,7 @@
         </is>
       </c>
       <c r="AU7" s="2" t="n"/>
+      <c r="AV7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2244,6 +2262,7 @@
         </is>
       </c>
       <c r="AU8" s="2" t="n"/>
+      <c r="AV8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2451,6 +2470,7 @@
         </is>
       </c>
       <c r="AU9" s="2" t="n"/>
+      <c r="AV9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -2664,6 +2684,7 @@
         </is>
       </c>
       <c r="AU10" s="8" t="n"/>
+      <c r="AV10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2873,6 +2894,7 @@
         </is>
       </c>
       <c r="AU11" s="2" t="n"/>
+      <c r="AV11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3088,6 +3110,7 @@
         </is>
       </c>
       <c r="AU12" s="2" t="n"/>
+      <c r="AV12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3303,6 +3326,11 @@
         </is>
       </c>
       <c r="AU13" s="2" t="inlineStr">
+        <is>
+          <t>치료기간 명시 없음. 자감초탕과 귀비탕 복용횟수 차이있음</t>
+        </is>
+      </c>
+      <c r="AV13" s="2" t="inlineStr">
         <is>
           <t>치료기간 명시 없음. 자감초탕과 귀비탕 복용횟수 차이있음</t>
         </is>

</xml_diff>